<commit_message>
Aprimora processo SAC e registro de atendimentos
</commit_message>
<xml_diff>
--- a/ERP_Portal_Fake/Sistema_Integrador_Portal_Fake/atendimentos_sac.xlsx
+++ b/ERP_Portal_Fake/Sistema_Integrador_Portal_Fake/atendimentos_sac.xlsx
@@ -511,7 +511,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>18/08/2026 13:53</t>
+          <t>18/08/2026 17:47</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -553,7 +553,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>FALHA</t>
+          <t>PENDENTE_CONTATO</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">

</xml_diff>

<commit_message>
feat: implementa processo 5 (relatórios, métricas, governança e versionamento)
</commit_message>
<xml_diff>
--- a/ERP_Portal_Fake/Sistema_Integrador_Portal_Fake/atendimentos_sac.xlsx
+++ b/ERP_Portal_Fake/Sistema_Integrador_Portal_Fake/atendimentos_sac.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -559,6 +559,58 @@
       <c r="J3" t="inlineStr">
         <is>
           <t>Cliente Hugo Lima não possui e-mail.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>PROT-20260818-152127-AE6793_CADASTRO_OK</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>PROT-20260818-152127-AE6793</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>03536054250</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Sannyer Nery</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026500534@ifam.edu.br</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>CONCLUIDO_P3</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>CADASTRO_OK</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>COMUNICADO</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>23/08/2026 19:06</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>E-mail enviado com sucesso.</t>
         </is>
       </c>
     </row>

</xml_diff>